<commit_message>
Complete Milestone 3: Project Intelligence and Risk Management
</commit_message>
<xml_diff>
--- a/Agile Documents/Defect_Tracker Template_v0.1 (1).xlsx
+++ b/Agile Documents/Defect_Tracker Template_v0.1 (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3ccdc670acfc4ce0/Desktop/Infosys Internship documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ai_Project_Intelligence_Risk_Advisor\Agile Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94A9FDE4-B2DE-4227-A871-8AAA440D75F4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E84AE3-EC24-46BD-ADCD-A597EBC6B89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="73">
   <si>
     <t>Submitted By</t>
   </si>
@@ -261,12 +261,66 @@
       <t xml:space="preserve"> package and verified the embedding model execution.</t>
     </r>
   </si>
+  <si>
+    <t>Documentation Generation Agent required generation of structured User Stories, Risk Register and Action Items from project documents.</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>Implemented the Documentation Generation Agent with RAG-based evidence retrieval and structured documentation generation.</t>
+  </si>
+  <si>
+    <t>Milestone 3 documentation generation functionality completed and validated.</t>
+  </si>
+  <si>
+    <t>Project required an automated health score to represent overall project condition using scope, timeline, risks and blockers.</t>
+  </si>
+  <si>
+    <t>Implemented the Project Health Scoring module with overall score and dimension-wise health evaluation.</t>
+  </si>
+  <si>
+    <t>Project health scoring integrated successfully into ProjectIQ.</t>
+  </si>
+  <si>
+    <t>Conversational assistant required evidence-grounded answers from uploaded project documents using RAG.</t>
+  </si>
+  <si>
+    <t>Integrated the RAG-based conversational Project Intelligence Assistant with uploaded project sources and local LLM.</t>
+  </si>
+  <si>
+    <t>Conversational project intelligence functionality completed and validated.</t>
+  </si>
+  <si>
+    <t>Assistant responses required improved retrieval for questions requesting complete lists such as objectives, deliverables and responsibilities.</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>Implemented enhanced multi-chunk retrieval with increased retrieval depth for list-based questions.</t>
+  </si>
+  <si>
+    <t>Retrieval improved to provide more complete project-specific responses.</t>
+  </si>
+  <si>
+    <t>Milestone 3 required validation of documentation outputs, health scoring and conversational assistant accuracy and relevance.</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>Performed end-to-end validation of Documentation Agent, Health Scoring module and RAG-based Conversational Assistant against uploaded project evidence.</t>
+  </si>
+  <si>
+    <t>Milestone 3 functionality validated and prepared for demonstration.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -363,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -392,6 +446,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,10 +464,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -701,7 +754,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="10" bestFit="1" customWidth="1"/>
@@ -710,13 +763,13 @@
     <col min="5" max="5" width="16" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" style="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.85546875" style="10" customWidth="1"/>
+    <col min="8" max="8" width="47.7109375" style="10" customWidth="1"/>
     <col min="9" max="10" width="21.85546875" style="11" customWidth="1"/>
     <col min="11" max="11" width="16.85546875" style="11" customWidth="1"/>
     <col min="12" max="16384" width="17.5703125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" ht="25.5">
+    <row r="1" spans="1:11" s="3" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
@@ -751,7 +804,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="76.5">
+    <row r="2" spans="1:11" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -786,7 +839,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="76.5">
+    <row r="3" spans="1:11" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -821,7 +874,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="51">
+    <row r="4" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -856,7 +909,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="63.75">
+    <row r="5" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -891,7 +944,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="51">
+    <row r="6" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -926,7 +979,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="78.75">
+    <row r="7" spans="1:11" ht="78.75" x14ac:dyDescent="0.2">
       <c r="A7" s="7">
         <v>1</v>
       </c>
@@ -961,7 +1014,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="78.75">
+    <row r="8" spans="1:11" ht="78.75" x14ac:dyDescent="0.2">
       <c r="A8" s="7">
         <v>2</v>
       </c>
@@ -996,7 +1049,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="110.25">
+    <row r="9" spans="1:11" ht="110.25" x14ac:dyDescent="0.2">
       <c r="A9" s="7">
         <v>3</v>
       </c>
@@ -1031,7 +1084,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="94.5">
+    <row r="10" spans="1:11" ht="94.5" x14ac:dyDescent="0.2">
       <c r="A10" s="7">
         <v>4</v>
       </c>
@@ -1066,7 +1119,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="78.75">
+    <row r="11" spans="1:11" ht="78.75" x14ac:dyDescent="0.2">
       <c r="A11" s="7">
         <v>5</v>
       </c>
@@ -1101,72 +1154,182 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" ht="15.75">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.75">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="15.75">
+    <row r="12" spans="1:11" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
+        <v>6</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="8">
+        <v>46290</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="I12" s="8">
+        <v>46290</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="7">
+        <v>7</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="8">
+        <v>46291</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I13" s="8">
+        <v>46291</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="7">
+        <v>8</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="8">
+        <v>46292</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" s="8">
+        <v>46292</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="7">
+        <v>9</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="8">
+        <v>46293</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="I15" s="8">
+        <v>46293</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="7">
+        <v>10</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="8">
+        <v>46294</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" s="8">
+        <v>46294</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="9"/>
@@ -1179,7 +1342,7 @@
       <c r="J17" s="9"/>
       <c r="K17" s="9"/>
     </row>
-    <row r="18" spans="1:11" ht="15.75">
+    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="9"/>
@@ -1192,7 +1355,7 @@
       <c r="J18" s="9"/>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="15.75">
+    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="9"/>
@@ -1228,29 +1391,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -1262,6 +1425,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1393,22 +1571,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1424,21 +1604,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>